<commit_message>
Wersja 2.5: odmiana złoty/złote/złotych w kwocie słownie
Kwota słownie na druku Delegacji odmienia jednostkę jak tysiące
(1 → złoty, 2–4 poza 12–14 → złote, reszta → złotych); przy ogółem = 0
pole zostaje puste. Sześć nowych testów; test.ps1 ponawia pobranie
kursów, gdy NBP chwilowo odrzuca zapytania.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wydanie/Kalkulator_delegacji_zagranicznej.xlsx
+++ b/wydanie/Kalkulator_delegacji_zagranicznej.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MOJE\Projekt_delegacje\wydanie\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF44211C-4F1B-475F-A67B-104D5F299A15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC67D37-767D-47A4-AC4C-79126AD2CD48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -291,7 +291,7 @@
     <t>Kontrola danych:</t>
   </si>
   <si>
-    <t>ver. 2.4 (09.10.2026) · wg rozporządzenia MPiPS z 29.01.2013 (t.j. Dz.U. 2023 poz. 2190) · kursy NBP pobierane automatycznie</t>
+    <t>ver. 2.5 (09.10.2026) · wg rozporządzenia MPiPS z 29.01.2013 (t.j. Dz.U. 2023 poz. 2190) · kursy NBP pobierane automatycznie</t>
   </si>
   <si>
     <t>Legenda:</t>
@@ -811,7 +811,7 @@
     <t>Jak korzystać z kalkulatora diety zagranicznej</t>
   </si>
   <si>
-    <t>Wersja 2.4 z 09.10.2026: kurs ręczny awaryjny; kontrola pustych etapów, posiłków i dat; druk delegacji (polecenie wyjazdu + rachunek kosztów), koszty przejazdów, noclegów i ryczałtów, kafelki z wynikiem, oznaczenie pól wymaganych i błędów, ochrona arkuszy.</t>
+    <t>Wersja 2.5 z 09.10.2026: kurs ręczny awaryjny; kontrola pustych etapów, posiłków i dat; druk delegacji (polecenie wyjazdu + rachunek kosztów), koszty przejazdów, noclegów i ryczałtów, kafelki z wynikiem, oznaczenie pól wymaganych i błędów, ochrona arkuszy.</t>
   </si>
   <si>
     <t>1. Arkusz „Kalkulator” – wypełniaj tylko żółte pola z niebieskim tekstem. Pozostałe komórki liczą się same.</t>
@@ -11513,7 +11513,7 @@
       <c r="G61" s="126"/>
       <c r="H61" s="127"/>
       <c r="I61" s="148" t="str" cm="1">
-        <f t="array" ref="I61">_xlfn.LET(_xlpm.x,ROUND(ABS(I60),2),_xlpm.z,INT(_xlpm.x),_xlpm.g,ROUND((_xlpm.x-_xlpm.z)*100,0),_xlpm.tri,_xlfn.LAMBDA(_xlpm.v,_xlfn.LET(_xlpm.h,INT(_xlpm.v/100),_xlpm.t,INT(MOD(_xlpm.v,100)/10),_xlpm.u,MOD(_xlpm.v,10),INDEX({"","sto","dwieście","trzysta","czterysta","pięćset","sześćset","siedemset","osiemset","dziewięćset"},_xlpm.h+1)&amp;" "&amp;IF(_xlpm.t=1,INDEX({"dziesięć","jedenaście","dwanaście","trzynaście","czternaście","piętnaście","szesnaście","siedemnaście","osiemnaście","dziewiętnaście"},_xlpm.u+1),INDEX({"","","dwadzieścia","trzydzieści","czterdzieści","pięćdziesiąt","sześćdziesiąt","siedemdziesiąt","osiemdziesiąt","dziewięćdziesiąt"},_xlpm.t+1)&amp;" "&amp;INDEX({"","jeden","dwa","trzy","cztery","pięć","sześć","siedem","osiem","dziewięć"},_xlpm.u+1)))),_xlpm.grp,_xlfn.LAMBDA(_xlpm.v,_xlpm.jd,_xlpm.dw,_xlpm.wl,IF(_xlpm.v=0,"",IF(_xlpm.v=1,_xlpm.jd,_xlpm.tri(_xlpm.v)&amp;" "&amp;IF(AND(MOD(_xlpm.v,10)&gt;=2,MOD(_xlpm.v,10)&lt;=4,OR(MOD(_xlpm.v,100)&lt;10,MOD(_xlpm.v,100)&gt;20)),_xlpm.dw,_xlpm.wl)))),_xlpm.s,TRIM(_xlpm.grp(INT(_xlpm.z/10^6),"jeden milion","miliony","milionów")&amp;" "&amp;_xlpm.grp(INT(MOD(_xlpm.z,10^6)/1000),"jeden tysiąc","tysiące","tysięcy")&amp;" "&amp;_xlpm.tri(MOD(_xlpm.z,1000))),IF(_xlpm.z=0,"zero",_xlpm.s)&amp;" złotych i "&amp;RIGHT("0"&amp;_xlpm.g,2)&amp;"/100")</f>
+        <f t="array" ref="I61">IF(N(I60)=0,"",_xlfn.LET(_xlpm.x,ROUND(ABS(I60),2),_xlpm.z,INT(_xlpm.x),_xlpm.g,ROUND((_xlpm.x-_xlpm.z)*100,0),_xlpm.tri,_xlfn.LAMBDA(_xlpm.v,_xlfn.LET(_xlpm.h,INT(_xlpm.v/100),_xlpm.t,INT(MOD(_xlpm.v,100)/10),_xlpm.u,MOD(_xlpm.v,10),INDEX({"","sto","dwieście","trzysta","czterysta","pięćset","sześćset","siedemset","osiemset","dziewięćset"},_xlpm.h+1)&amp;" "&amp;IF(_xlpm.t=1,INDEX({"dziesięć","jedenaście","dwanaście","trzynaście","czternaście","piętnaście","szesnaście","siedemnaście","osiemnaście","dziewiętnaście"},_xlpm.u+1),INDEX({"","","dwadzieścia","trzydzieści","czterdzieści","pięćdziesiąt","sześćdziesiąt","siedemdziesiąt","osiemdziesiąt","dziewięćdziesiąt"},_xlpm.t+1)&amp;" "&amp;INDEX({"","jeden","dwa","trzy","cztery","pięć","sześć","siedem","osiem","dziewięć"},_xlpm.u+1)))),_xlpm.grp,_xlfn.LAMBDA(_xlpm.v,_xlpm.jd,_xlpm.dw,_xlpm.wl,IF(_xlpm.v=0,"",IF(_xlpm.v=1,_xlpm.jd,_xlpm.tri(_xlpm.v)&amp;" "&amp;IF(AND(MOD(_xlpm.v,10)&gt;=2,MOD(_xlpm.v,10)&lt;=4,OR(MOD(_xlpm.v,100)&lt;10,MOD(_xlpm.v,100)&gt;20)),_xlpm.dw,_xlpm.wl)))),_xlpm.s,TRIM(_xlpm.grp(INT(_xlpm.z/10^6),"jeden milion","miliony","milionów")&amp;" "&amp;_xlpm.grp(INT(MOD(_xlpm.z,10^6)/1000),"jeden tysiąc","tysiące","tysięcy")&amp;" "&amp;_xlpm.tri(MOD(_xlpm.z,1000))),IF(_xlpm.z=0,"zero",_xlpm.s)&amp;" "&amp;IF(_xlpm.z=1,"złoty i",IF(AND(MOD(_xlpm.z,10)&gt;=2,MOD(_xlpm.z,10)&lt;=4,OR(MOD(_xlpm.z,100)&lt;10,MOD(_xlpm.z,100)&gt;20)),"złote i","złotych i"))&amp;" "&amp;RIGHT("0"&amp;_xlpm.g,2)&amp;"/100"))</f>
         <v>dwa tysiące pięćset siedemdziesiąt złotych i 96/100</v>
       </c>
       <c r="J61" s="1"/>

</xml_diff>